<commit_message>
Update Agile documents for Milestone 2
</commit_message>
<xml_diff>
--- a/docs/Defect_Tracker Template_v0.1 (1).xlsx
+++ b/docs/Defect_Tracker Template_v0.1 (1).xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="53">
   <si>
     <t>Sl No</t>
   </si>
@@ -122,6 +122,63 @@
   </si>
   <si>
     <t>Generated uploads and knowledge-base files could be added to Git repository.</t>
+  </si>
+  <si>
+    <t>16/09/2026</t>
+  </si>
+  <si>
+    <t>DOCX milestone tables were not extracted by the document loader, causing milestone information to be missing from the agent context.</t>
+  </si>
+  <si>
+    <t>Data Extraction</t>
+  </si>
+  <si>
+    <t>Updated DOCX loader to extract both paragraphs and table contents.</t>
+  </si>
+  <si>
+    <t>Verified with project plan containing milestone table.</t>
+  </si>
+  <si>
+    <t>Scope Extraction Agent returned an empty responsibilities list even when responsibility information was present in the retrieved context.</t>
+  </si>
+  <si>
+    <t>Updated scope extraction prompt and tested responsibility extraction with project documents.</t>
+  </si>
+  <si>
+    <t>Open</t>
+  </si>
+  <si>
+    <t>Requires additional validation with multiple documents.</t>
+  </si>
+  <si>
+    <t>Blocker Agent incorrectly classified the final project deadline as a pending decision.</t>
+  </si>
+  <si>
+    <t>Strengthened pending-decision rules to accept only explicitly unresolved decisions.</t>
+  </si>
+  <si>
+    <t>Further testing required to prevent incorrect classification.</t>
+  </si>
+  <si>
+    <t>Blocker Agent inferred a due date for an action item from a milestone date instead of using an explicitly stated action-item due date.</t>
+  </si>
+  <si>
+    <t>Updated agent instructions to avoid inventing or inferring action-item due dates.</t>
+  </si>
+  <si>
+    <t>Validate using meeting-notes documents.</t>
+  </si>
+  <si>
+    <t>Local Ollama LLM response generation was significantly slower than the previously used OpenAI API.</t>
+  </si>
+  <si>
+    <t>Performance</t>
+  </si>
+  <si>
+    <t>Migrated LLM execution from OpenAI API to local Ollama after API credits were exhausted. Performance optimization is pending.</t>
+  </si>
+  <si>
+    <t>Local model provides usable responses but requires optimization.</t>
   </si>
 </sst>
 </file>
@@ -781,69 +838,179 @@
       </c>
     </row>
     <row r="7" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="6"/>
+      <c r="A7" s="5">
+        <v>6</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E7" s="3">
+        <v>2</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="8" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
+      <c r="A8" s="3">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" s="3">
+        <v>2</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="9" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="6"/>
+      <c r="A9" s="5">
+        <v>8</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" s="3">
+        <v>2</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="10" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="6"/>
+      <c r="A10" s="5">
+        <v>9</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E10" s="3">
+        <v>2</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="11" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
+      <c r="A11" s="3">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E11" s="3">
+        <v>2</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="12" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="5"/>
@@ -1025,15 +1192,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F50FC49184C87E449886FB52439922C9" ma:contentTypeVersion="2" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f85b7e58c3d8889ba0673e7b34a193a6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b67b99c0-208c-4860-83e0-51466af787c4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5d43477c1ade21a66d9a75ba2d5aa042" ns2:_="">
     <xsd:import namespace="b67b99c0-208c-4860-83e0-51466af787c4"/>
@@ -1165,6 +1323,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
   <ds:schemaRefs>
@@ -1175,14 +1342,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{191CB444-B9BF-4C91-94BD-600524521497}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1198,4 +1357,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>